<commit_message>
Update project layout and code
</commit_message>
<xml_diff>
--- a/dataset.xlsx
+++ b/dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\multimodal_ai_hackathon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F49290DB-757D-4D4C-9E24-782196582C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A73E2F1-8B55-4B76-8E30-BE0CEE67DE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2468,7 +2468,9 @@
     <col min="5" max="5" width="11.3984375" style="1" customWidth="1"/>
     <col min="6" max="6" width="23.69921875" style="1" customWidth="1"/>
     <col min="7" max="7" width="25.19921875" style="1" customWidth="1"/>
-    <col min="8" max="11" width="10.19921875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="27.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.69921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.19921875" style="1" customWidth="1"/>
     <col min="12" max="12" width="12.09765625" style="1" customWidth="1"/>
     <col min="13" max="13" width="34.19921875" style="1" customWidth="1"/>
     <col min="14" max="14" width="16.8984375" style="1" customWidth="1"/>
@@ -2480,12 +2482,12 @@
     <col min="20" max="20" width="18.3984375" style="1" customWidth="1"/>
     <col min="21" max="21" width="21.5" style="1" customWidth="1"/>
     <col min="22" max="22" width="18.3984375" style="1" customWidth="1"/>
-    <col min="23" max="23" width="13.59765625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="28.5" style="1" customWidth="1"/>
     <col min="24" max="24" width="10.19921875" style="1" customWidth="1"/>
-    <col min="25" max="25" width="13.19921875" style="1" customWidth="1"/>
+    <col min="25" max="25" width="30.8984375" style="1" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="19.09765625" style="1" customWidth="1"/>
     <col min="27" max="27" width="21.69921875" style="1" customWidth="1"/>
-    <col min="28" max="28" width="17.8984375" style="1" customWidth="1"/>
+    <col min="28" max="28" width="25" style="1" customWidth="1"/>
     <col min="29" max="29" width="10.19921875" style="1" customWidth="1"/>
     <col min="30" max="30" width="29.5" style="1" customWidth="1"/>
     <col min="31" max="37" width="10.19921875" style="1" customWidth="1"/>

</xml_diff>